<commit_message>
Perbaiki NIP Adams Resmitha Thalib dan hapus permanen 3 staf resign
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Clustering-Akun-LokaKin.xlsx
+++ b/Clustering-Akun-LokaKin.xlsx
@@ -2156,7 +2156,11 @@
           <t>Adams Resmitha Thalib, SE</t>
         </is>
       </c>
-      <c r="D43" s="5" t="n"/>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>198305192025211000</t>
+        </is>
+      </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
           <t>Layanan Rehabilitasi Sosial</t>
@@ -2175,11 +2179,7 @@
         <v>1</v>
       </c>
       <c r="L43" s="5" t="inlineStr"/>
-      <c r="M43" s="5" t="inlineStr">
-        <is>
-          <t>NIP/NIK belum ada — wajib diisi agar akun dapat login.</t>
-        </is>
-      </c>
+      <c r="M43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -5827,7 +5827,11 @@
           <t>Adams Resmitha Thalib, SE</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr"/>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>198305192025211000</t>
+        </is>
+      </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
           <t>staff</t>
@@ -5851,12 +5855,12 @@
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>roster-sync</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-10-21T14:49:04</t>
         </is>
       </c>
     </row>

</xml_diff>